<commit_message>
Add June budget application email draft
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2026/PP-2606 Monthly Budget Application Form.xlsx
+++ b/2026/PP-2606 Monthly Budget Application Form.xlsx
@@ -5802,7 +5802,7 @@
       </c>
       <c r="E11" s="138">
         <f t="shared" si="2">SUM(E4:E10)</f>
-        <v>63872.76</v>
+        <v>53872.76</v>
       </c>
       <c r="F11" s="138">
         <f t="shared" si="2"/>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="H11" s="141">
         <f t="shared" si="2">SUM(H4:H10)</f>
-        <v>82585.76</v>
+        <v>72585.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>